<commit_message>
Use Clang 14 as baseline in plots
</commit_message>
<xml_diff>
--- a/data/git/file/git.o.xlsx
+++ b/data/git/file/git.o.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/jryans/Research/Papers/oopsla-2023/data/git/file/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F4EE94F-1886-AC42-99FA-F241CAEFF560}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E3B8E25-D8A3-F845-B160-26E10E7F6B7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="16440" yWindow="1920" windowWidth="47060" windowHeight="24880" activeTab="2" xr2:uid="{1069CAA2-7C27-E54E-B88A-C9343E41429C}"/>
+    <workbookView xWindow="16440" yWindow="1920" windowWidth="47060" windowHeight="24880" activeTab="1" xr2:uid="{1069CAA2-7C27-E54E-B88A-C9343E41429C}"/>
   </bookViews>
   <sheets>
     <sheet name="Wide" sheetId="1" r:id="rId1"/>
@@ -658,9 +658,6 @@
     <t>O1-14 Delta</t>
   </si>
   <si>
-    <t xml:space="preserve">CL / SL (O0-13, m2r)    </t>
-  </si>
-  <si>
     <t>CL / SL (O1-12)</t>
   </si>
   <si>
@@ -673,9 +670,6 @@
     <t>CL / SL Delta</t>
   </si>
   <si>
-    <t>CL (O0-13, m2r)</t>
-  </si>
-  <si>
     <t>CL (O1-12)</t>
   </si>
   <si>
@@ -683,24 +677,6 @@
   </si>
   <si>
     <t>CL (O1-14)</t>
-  </si>
-  <si>
-    <t>CL / SL (O0-13)</t>
-  </si>
-  <si>
-    <t>CL (O0-13)</t>
-  </si>
-  <si>
-    <t>Clang 13, O0</t>
-  </si>
-  <si>
-    <t>O0-13 Delta</t>
-  </si>
-  <si>
-    <t>O0-13, m2r Delta</t>
-  </si>
-  <si>
-    <t>Clang 13, O0 + mem2reg</t>
   </si>
   <si>
     <t>Arithmetic Mean (Normalised)</t>
@@ -717,14 +693,45 @@
   <si>
     <t>Clang 14, O2</t>
   </si>
+  <si>
+    <t>CL / SL (O0-14)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CL / SL (O0-14, m2r)    </t>
+  </si>
+  <si>
+    <t>O0-14 Delta</t>
+  </si>
+  <si>
+    <t>O0-14, m2r Delta</t>
+  </si>
+  <si>
+    <t>CL (O0-14)</t>
+  </si>
+  <si>
+    <t>CL (O0-14, m2r)</t>
+  </si>
+  <si>
+    <t>Clang 14, O0</t>
+  </si>
+  <si>
+    <t>Clang 14, O0 + mem2reg</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="11" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -814,10 +821,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -853,59 +861,59 @@
 </file>
 
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_6" connectionId="17" xr16:uid="{BF097535-9BC4-8A44-8028-889020E90CD1}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_4" connectionId="15" xr16:uid="{12472C14-9457-0C4B-85A7-6B4E9A0A4A3A}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable10.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_3" connectionId="14" xr16:uid="{ED71FF77-6ABC-D749-8E21-C2BBC0C49B38}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_2" connectionId="13" xr16:uid="{577EB844-CFFF-874E-B636-A682F7CA9C09}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable11.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_10" connectionId="12" xr16:uid="{6F5AE438-0047-EF40-9065-31B57EBCFEA0}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_9" connectionId="20" xr16:uid="{DF99720B-8FB8-1945-B82B-62174EC5794B}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable12.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_9" connectionId="20" xr16:uid="{DF99720B-8FB8-1945-B82B-62174EC5794B}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O013m2r" connectionId="2" xr16:uid="{9CCAF8A0-2B7D-0548-BCF8-D231422B6B5F}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable13.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O113" connectionId="7" xr16:uid="{7EC8FDAA-8641-7F44-A40C-DFADA06143DC}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable14.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O114" connectionId="9" xr16:uid="{6DA84D36-F075-D643-87AE-9205D8C2E13B}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable15.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O013m2r" connectionId="3" xr16:uid="{6BD7D553-8716-684F-A112-947029E7B50E}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable16.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O112" connectionId="5" xr16:uid="{5C22DE01-5C44-7C4E-9EAF-E54F03689DF7}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable14.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O113" connectionId="7" xr16:uid="{7EC8FDAA-8641-7F44-A40C-DFADA06143DC}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<file path=xl/queryTables/queryTable17.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O112" connectionId="6" xr16:uid="{72FE5272-0C81-7B49-8C92-9E8FE63CCD65}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable15.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O114" connectionId="9" xr16:uid="{6DA84D36-F075-D643-87AE-9205D8C2E13B}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<file path=xl/queryTables/queryTable18.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O013m2r" connectionId="4" xr16:uid="{F1095D83-ED7E-9549-9DFC-EB98E00E3997}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable16.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O013m2r" connectionId="3" xr16:uid="{6BD7D553-8716-684F-A112-947029E7B50E}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<file path=xl/queryTables/queryTable19.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O114" connectionId="10" xr16:uid="{D34FF5A8-62F7-554D-9E92-8F5C8D099217}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_5" connectionId="16" xr16:uid="{5AF1A4D8-20C7-B944-973B-C6F106978454}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable20.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O113" connectionId="8" xr16:uid="{061FB766-530C-7F46-AA03-8A3221BEEC32}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable18.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O112" connectionId="6" xr16:uid="{72FE5272-0C81-7B49-8C92-9E8FE63CCD65}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
-<file path=xl/queryTables/queryTable19.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O013m2r" connectionId="4" xr16:uid="{F1095D83-ED7E-9549-9DFC-EB98E00E3997}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
-<file path=xl/queryTables/queryTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_2" connectionId="13" xr16:uid="{577EB844-CFFF-874E-B636-A682F7CA9C09}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
-<file path=xl/queryTables/queryTable20.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O114" connectionId="10" xr16:uid="{D34FF5A8-62F7-554D-9E92-8F5C8D099217}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
 <file path=xl/queryTables/queryTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_4" connectionId="15" xr16:uid="{12472C14-9457-0C4B-85A7-6B4E9A0A4A3A}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_7" connectionId="18" xr16:uid="{D6E8256A-0710-A34A-80B4-71635A8A7FF9}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/queryTables/queryTable4.xml><?xml version="1.0" encoding="utf-8"?>
@@ -913,23 +921,23 @@
 </file>
 
 <file path=xl/queryTables/queryTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_3" connectionId="14" xr16:uid="{ED71FF77-6ABC-D749-8E21-C2BBC0C49B38}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_1" connectionId="11" xr16:uid="{3FDFE62B-64A1-F14C-AAB6-88B8E3E9B697}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/queryTables/queryTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_10" connectionId="12" xr16:uid="{6F5AE438-0047-EF40-9065-31B57EBCFEA0}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+</file>
+
+<file path=xl/queryTables/queryTable8.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_8" connectionId="19" xr16:uid="{6528BD19-FD94-5B40-8D88-624F75163B95}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
-<file path=xl/queryTables/queryTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o.O013m2r" connectionId="2" xr16:uid="{9CCAF8A0-2B7D-0548-BCF8-D231422B6B5F}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
-<file path=xl/queryTables/queryTable8.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_5" connectionId="16" xr16:uid="{5AF1A4D8-20C7-B944-973B-C6F106978454}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
-</file>
-
 <file path=xl/queryTables/queryTable9.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_7" connectionId="18" xr16:uid="{D6E8256A-0710-A34A-80B4-71635A8A7FF9}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
+<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="git.o_6" connectionId="17" xr16:uid="{BF097535-9BC4-8A44-8028-889020E90CD1}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="1" applyPatternFormats="1" applyAlignmentFormats="0" applyWidthHeightFormats="0"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1255,31 +1263,31 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>109</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>111</v>
+      </c>
+      <c r="G1" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="C1" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="D1" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="E1" s="2" t="s">
-        <v>111</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="G1" s="2" t="s">
-        <v>126</v>
-      </c>
       <c r="H1" s="2" t="s">
-        <v>127</v>
+        <v>119</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="K1" s="2" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="L1" s="2" t="s">
         <v>106</v>
@@ -1291,19 +1299,19 @@
         <v>108</v>
       </c>
       <c r="P1" s="2" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="Q1" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="R1" s="2" t="s">
+        <v>113</v>
+      </c>
+      <c r="S1" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="R1" s="2" t="s">
+      <c r="T1" s="2" t="s">
         <v>115</v>
-      </c>
-      <c r="S1" s="2" t="s">
-        <v>116</v>
-      </c>
-      <c r="T1" s="2" t="s">
-        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:20" x14ac:dyDescent="0.25">
@@ -7433,15 +7441,15 @@
         <v>102</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>125</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A2" s="7" t="s">
-        <v>120</v>
+      <c r="A2" s="9" t="s">
+        <v>127</v>
       </c>
       <c r="B2" s="7">
         <f>1+AVERAGE(Wide!J2:J101)</f>
@@ -7457,8 +7465,8 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
-      <c r="A3" s="7" t="s">
-        <v>123</v>
+      <c r="A3" s="9" t="s">
+        <v>128</v>
       </c>
       <c r="B3" s="7">
         <f>1+AVERAGE(Wide!K2:K101)</f>
@@ -7525,7 +7533,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -7557,7 +7565,7 @@
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B2" s="3" t="s">
         <v>29</v>
@@ -7569,7 +7577,7 @@
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>83</v>
@@ -7581,7 +7589,7 @@
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>84</v>
@@ -7593,7 +7601,7 @@
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B5" s="3" t="s">
         <v>85</v>
@@ -7605,7 +7613,7 @@
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B6" s="3" t="s">
         <v>86</v>
@@ -7617,7 +7625,7 @@
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B7" s="3" t="s">
         <v>87</v>
@@ -7629,7 +7637,7 @@
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B8" s="3" t="s">
         <v>88</v>
@@ -7641,7 +7649,7 @@
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>25</v>
@@ -7653,7 +7661,7 @@
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B10" s="3" t="s">
         <v>27</v>
@@ -7665,7 +7673,7 @@
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>28</v>
@@ -7677,7 +7685,7 @@
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B12" s="3" t="s">
         <v>26</v>
@@ -7689,7 +7697,7 @@
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>36</v>
@@ -7701,7 +7709,7 @@
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>35</v>
@@ -7713,7 +7721,7 @@
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>5</v>
@@ -7725,7 +7733,7 @@
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B16" s="3" t="s">
         <v>6</v>
@@ -7737,7 +7745,7 @@
     </row>
     <row r="17" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>7</v>
@@ -7749,7 +7757,7 @@
     </row>
     <row r="18" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B18" s="3" t="s">
         <v>31</v>
@@ -7761,7 +7769,7 @@
     </row>
     <row r="19" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>32</v>
@@ -7773,7 +7781,7 @@
     </row>
     <row r="20" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B20" s="3" t="s">
         <v>30</v>
@@ -7785,7 +7793,7 @@
     </row>
     <row r="21" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>100</v>
@@ -7797,7 +7805,7 @@
     </row>
     <row r="22" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B22" s="3" t="s">
         <v>67</v>
@@ -7809,7 +7817,7 @@
     </row>
     <row r="23" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B23" s="3" t="s">
         <v>66</v>
@@ -7821,7 +7829,7 @@
     </row>
     <row r="24" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B24" s="3" t="s">
         <v>78</v>
@@ -7833,7 +7841,7 @@
     </row>
     <row r="25" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B25" s="3" t="s">
         <v>79</v>
@@ -7845,7 +7853,7 @@
     </row>
     <row r="26" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B26" s="3" t="s">
         <v>71</v>
@@ -7857,7 +7865,7 @@
     </row>
     <row r="27" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B27" s="3" t="s">
         <v>72</v>
@@ -7869,7 +7877,7 @@
     </row>
     <row r="28" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B28" s="3" t="s">
         <v>81</v>
@@ -7881,7 +7889,7 @@
     </row>
     <row r="29" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B29" s="3" t="s">
         <v>74</v>
@@ -7893,7 +7901,7 @@
     </row>
     <row r="30" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B30" s="3" t="s">
         <v>73</v>
@@ -7905,7 +7913,7 @@
     </row>
     <row r="31" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B31" s="3" t="s">
         <v>75</v>
@@ -7917,7 +7925,7 @@
     </row>
     <row r="32" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B32" s="3" t="s">
         <v>82</v>
@@ -7929,7 +7937,7 @@
     </row>
     <row r="33" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B33" s="3" t="s">
         <v>80</v>
@@ -7941,7 +7949,7 @@
     </row>
     <row r="34" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B34" s="3" t="s">
         <v>76</v>
@@ -7953,7 +7961,7 @@
     </row>
     <row r="35" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B35" s="3" t="s">
         <v>77</v>
@@ -7965,7 +7973,7 @@
     </row>
     <row r="36" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B36" s="3" t="s">
         <v>15</v>
@@ -7977,7 +7985,7 @@
     </row>
     <row r="37" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B37" s="3" t="s">
         <v>17</v>
@@ -7989,7 +7997,7 @@
     </row>
     <row r="38" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B38" s="3" t="s">
         <v>16</v>
@@ -8001,7 +8009,7 @@
     </row>
     <row r="39" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B39" s="3" t="s">
         <v>19</v>
@@ -8013,7 +8021,7 @@
     </row>
     <row r="40" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B40" s="3" t="s">
         <v>18</v>
@@ -8025,7 +8033,7 @@
     </row>
     <row r="41" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B41" s="3" t="s">
         <v>20</v>
@@ -8037,7 +8045,7 @@
     </row>
     <row r="42" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B42" s="3" t="s">
         <v>90</v>
@@ -8049,7 +8057,7 @@
     </row>
     <row r="43" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B43" s="3" t="s">
         <v>89</v>
@@ -8061,7 +8069,7 @@
     </row>
     <row r="44" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B44" s="3" t="s">
         <v>93</v>
@@ -8073,7 +8081,7 @@
     </row>
     <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B45" s="3" t="s">
         <v>94</v>
@@ -8085,7 +8093,7 @@
     </row>
     <row r="46" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B46" s="3" t="s">
         <v>91</v>
@@ -8097,7 +8105,7 @@
     </row>
     <row r="47" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B47" s="3" t="s">
         <v>96</v>
@@ -8109,7 +8117,7 @@
     </row>
     <row r="48" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B48" s="3" t="s">
         <v>95</v>
@@ -8121,7 +8129,7 @@
     </row>
     <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B49" s="3" t="s">
         <v>92</v>
@@ -8133,7 +8141,7 @@
     </row>
     <row r="50" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B50" s="3" t="s">
         <v>99</v>
@@ -8145,7 +8153,7 @@
     </row>
     <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B51" s="3" t="s">
         <v>64</v>
@@ -8157,7 +8165,7 @@
     </row>
     <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B52" s="3" t="s">
         <v>65</v>
@@ -8169,7 +8177,7 @@
     </row>
     <row r="53" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B53" s="3" t="s">
         <v>63</v>
@@ -8181,7 +8189,7 @@
     </row>
     <row r="54" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B54" s="3" t="s">
         <v>11</v>
@@ -8193,7 +8201,7 @@
     </row>
     <row r="55" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B55" s="3" t="s">
         <v>13</v>
@@ -8205,7 +8213,7 @@
     </row>
     <row r="56" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B56" s="3" t="s">
         <v>9</v>
@@ -8217,7 +8225,7 @@
     </row>
     <row r="57" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B57" s="3" t="s">
         <v>10</v>
@@ -8229,7 +8237,7 @@
     </row>
     <row r="58" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B58" s="3" t="s">
         <v>14</v>
@@ -8241,7 +8249,7 @@
     </row>
     <row r="59" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B59" s="3" t="s">
         <v>12</v>
@@ -8253,7 +8261,7 @@
     </row>
     <row r="60" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B60" s="3" t="s">
         <v>8</v>
@@ -8265,7 +8273,7 @@
     </row>
     <row r="61" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B61" s="3" t="s">
         <v>60</v>
@@ -8277,7 +8285,7 @@
     </row>
     <row r="62" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B62" s="3" t="s">
         <v>62</v>
@@ -8289,7 +8297,7 @@
     </row>
     <row r="63" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B63" s="3" t="s">
         <v>61</v>
@@ -8301,7 +8309,7 @@
     </row>
     <row r="64" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B64" s="3" t="s">
         <v>59</v>
@@ -8313,7 +8321,7 @@
     </row>
     <row r="65" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B65" s="3" t="s">
         <v>2</v>
@@ -8325,7 +8333,7 @@
     </row>
     <row r="66" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B66" s="3" t="s">
         <v>1</v>
@@ -8337,7 +8345,7 @@
     </row>
     <row r="67" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B67" s="3" t="s">
         <v>3</v>
@@ -8349,7 +8357,7 @@
     </row>
     <row r="68" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B68" s="3" t="s">
         <v>4</v>
@@ -8361,7 +8369,7 @@
     </row>
     <row r="69" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B69" s="3" t="s">
         <v>21</v>
@@ -8373,7 +8381,7 @@
     </row>
     <row r="70" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B70" s="3" t="s">
         <v>23</v>
@@ -8385,7 +8393,7 @@
     </row>
     <row r="71" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B71" s="3" t="s">
         <v>24</v>
@@ -8397,7 +8405,7 @@
     </row>
     <row r="72" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B72" s="3" t="s">
         <v>22</v>
@@ -8409,7 +8417,7 @@
     </row>
     <row r="73" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B73" s="3" t="s">
         <v>40</v>
@@ -8421,7 +8429,7 @@
     </row>
     <row r="74" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B74" s="3" t="s">
         <v>41</v>
@@ -8433,7 +8441,7 @@
     </row>
     <row r="75" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B75" s="3" t="s">
         <v>45</v>
@@ -8445,7 +8453,7 @@
     </row>
     <row r="76" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B76" s="3" t="s">
         <v>42</v>
@@ -8457,7 +8465,7 @@
     </row>
     <row r="77" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B77" s="3" t="s">
         <v>43</v>
@@ -8469,7 +8477,7 @@
     </row>
     <row r="78" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B78" s="3" t="s">
         <v>46</v>
@@ -8481,7 +8489,7 @@
     </row>
     <row r="79" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B79" s="3" t="s">
         <v>48</v>
@@ -8493,7 +8501,7 @@
     </row>
     <row r="80" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B80" s="3" t="s">
         <v>49</v>
@@ -8505,7 +8513,7 @@
     </row>
     <row r="81" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B81" s="3" t="s">
         <v>47</v>
@@ -8517,7 +8525,7 @@
     </row>
     <row r="82" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B82" s="3" t="s">
         <v>44</v>
@@ -8529,7 +8537,7 @@
     </row>
     <row r="83" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B83" s="3" t="s">
         <v>51</v>
@@ -8541,7 +8549,7 @@
     </row>
     <row r="84" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B84" s="3" t="s">
         <v>52</v>
@@ -8553,7 +8561,7 @@
     </row>
     <row r="85" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B85" s="3" t="s">
         <v>55</v>
@@ -8565,7 +8573,7 @@
     </row>
     <row r="86" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B86" s="3" t="s">
         <v>58</v>
@@ -8577,7 +8585,7 @@
     </row>
     <row r="87" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B87" s="3" t="s">
         <v>50</v>
@@ -8589,7 +8597,7 @@
     </row>
     <row r="88" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B88" s="3" t="s">
         <v>56</v>
@@ -8601,7 +8609,7 @@
     </row>
     <row r="89" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B89" s="3" t="s">
         <v>54</v>
@@ -8613,7 +8621,7 @@
     </row>
     <row r="90" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B90" s="3" t="s">
         <v>53</v>
@@ -8625,7 +8633,7 @@
     </row>
     <row r="91" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B91" s="3" t="s">
         <v>57</v>
@@ -8637,7 +8645,7 @@
     </row>
     <row r="92" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B92" s="3" t="s">
         <v>33</v>
@@ -8649,7 +8657,7 @@
     </row>
     <row r="93" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B93" s="3" t="s">
         <v>34</v>
@@ -8661,7 +8669,7 @@
     </row>
     <row r="94" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B94" s="3" t="s">
         <v>70</v>
@@ -8673,7 +8681,7 @@
     </row>
     <row r="95" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B95" s="3" t="s">
         <v>69</v>
@@ -8685,7 +8693,7 @@
     </row>
     <row r="96" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B96" s="3" t="s">
         <v>68</v>
@@ -8697,7 +8705,7 @@
     </row>
     <row r="97" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B97" s="3" t="s">
         <v>37</v>
@@ -8709,7 +8717,7 @@
     </row>
     <row r="98" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B98" s="3" t="s">
         <v>38</v>
@@ -8721,7 +8729,7 @@
     </row>
     <row r="99" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B99" s="3" t="s">
         <v>98</v>
@@ -8733,7 +8741,7 @@
     </row>
     <row r="100" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B100" s="3" t="s">
         <v>97</v>
@@ -8745,7 +8753,7 @@
     </row>
     <row r="101" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B101" s="3" t="s">
         <v>39</v>
@@ -8757,7 +8765,7 @@
     </row>
     <row r="102" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A102" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B102" s="3" t="s">
         <v>29</v>
@@ -8769,7 +8777,7 @@
     </row>
     <row r="103" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B103" s="3" t="s">
         <v>83</v>
@@ -8781,7 +8789,7 @@
     </row>
     <row r="104" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B104" s="3" t="s">
         <v>84</v>
@@ -8793,7 +8801,7 @@
     </row>
     <row r="105" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B105" s="3" t="s">
         <v>85</v>
@@ -8805,7 +8813,7 @@
     </row>
     <row r="106" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B106" s="3" t="s">
         <v>86</v>
@@ -8817,7 +8825,7 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B107" s="3" t="s">
         <v>87</v>
@@ -8829,7 +8837,7 @@
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B108" s="3" t="s">
         <v>88</v>
@@ -8841,7 +8849,7 @@
     </row>
     <row r="109" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B109" s="3" t="s">
         <v>25</v>
@@ -8853,7 +8861,7 @@
     </row>
     <row r="110" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B110" s="3" t="s">
         <v>27</v>
@@ -8865,7 +8873,7 @@
     </row>
     <row r="111" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B111" s="3" t="s">
         <v>28</v>
@@ -8877,7 +8885,7 @@
     </row>
     <row r="112" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B112" s="3" t="s">
         <v>26</v>
@@ -8889,7 +8897,7 @@
     </row>
     <row r="113" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B113" s="3" t="s">
         <v>36</v>
@@ -8901,7 +8909,7 @@
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B114" s="3" t="s">
         <v>35</v>
@@ -8913,7 +8921,7 @@
     </row>
     <row r="115" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B115" s="3" t="s">
         <v>5</v>
@@ -8925,7 +8933,7 @@
     </row>
     <row r="116" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B116" s="3" t="s">
         <v>6</v>
@@ -8937,7 +8945,7 @@
     </row>
     <row r="117" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B117" s="3" t="s">
         <v>7</v>
@@ -8949,7 +8957,7 @@
     </row>
     <row r="118" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B118" s="3" t="s">
         <v>31</v>
@@ -8961,7 +8969,7 @@
     </row>
     <row r="119" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B119" s="3" t="s">
         <v>32</v>
@@ -8973,7 +8981,7 @@
     </row>
     <row r="120" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B120" s="3" t="s">
         <v>30</v>
@@ -8985,7 +8993,7 @@
     </row>
     <row r="121" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B121" s="3" t="s">
         <v>100</v>
@@ -8997,7 +9005,7 @@
     </row>
     <row r="122" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B122" s="3" t="s">
         <v>67</v>
@@ -9009,7 +9017,7 @@
     </row>
     <row r="123" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B123" s="3" t="s">
         <v>66</v>
@@ -9021,7 +9029,7 @@
     </row>
     <row r="124" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B124" s="3" t="s">
         <v>78</v>
@@ -9033,7 +9041,7 @@
     </row>
     <row r="125" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B125" s="3" t="s">
         <v>79</v>
@@ -9045,7 +9053,7 @@
     </row>
     <row r="126" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B126" s="3" t="s">
         <v>71</v>
@@ -9057,7 +9065,7 @@
     </row>
     <row r="127" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B127" s="3" t="s">
         <v>72</v>
@@ -9069,7 +9077,7 @@
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B128" s="3" t="s">
         <v>81</v>
@@ -9081,7 +9089,7 @@
     </row>
     <row r="129" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B129" s="3" t="s">
         <v>74</v>
@@ -9093,7 +9101,7 @@
     </row>
     <row r="130" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B130" s="3" t="s">
         <v>73</v>
@@ -9105,7 +9113,7 @@
     </row>
     <row r="131" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B131" s="3" t="s">
         <v>75</v>
@@ -9117,7 +9125,7 @@
     </row>
     <row r="132" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B132" s="3" t="s">
         <v>82</v>
@@ -9129,7 +9137,7 @@
     </row>
     <row r="133" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B133" s="3" t="s">
         <v>80</v>
@@ -9141,7 +9149,7 @@
     </row>
     <row r="134" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B134" s="3" t="s">
         <v>76</v>
@@ -9153,7 +9161,7 @@
     </row>
     <row r="135" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B135" s="3" t="s">
         <v>77</v>
@@ -9165,7 +9173,7 @@
     </row>
     <row r="136" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B136" s="3" t="s">
         <v>15</v>
@@ -9177,7 +9185,7 @@
     </row>
     <row r="137" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B137" s="3" t="s">
         <v>17</v>
@@ -9189,7 +9197,7 @@
     </row>
     <row r="138" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B138" s="3" t="s">
         <v>16</v>
@@ -9201,7 +9209,7 @@
     </row>
     <row r="139" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B139" s="3" t="s">
         <v>19</v>
@@ -9213,7 +9221,7 @@
     </row>
     <row r="140" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B140" s="3" t="s">
         <v>18</v>
@@ -9225,7 +9233,7 @@
     </row>
     <row r="141" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B141" s="3" t="s">
         <v>20</v>
@@ -9237,7 +9245,7 @@
     </row>
     <row r="142" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B142" s="3" t="s">
         <v>90</v>
@@ -9249,7 +9257,7 @@
     </row>
     <row r="143" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A143" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B143" s="3" t="s">
         <v>89</v>
@@ -9261,7 +9269,7 @@
     </row>
     <row r="144" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B144" s="3" t="s">
         <v>93</v>
@@ -9273,7 +9281,7 @@
     </row>
     <row r="145" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B145" s="3" t="s">
         <v>94</v>
@@ -9285,7 +9293,7 @@
     </row>
     <row r="146" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B146" s="3" t="s">
         <v>91</v>
@@ -9297,7 +9305,7 @@
     </row>
     <row r="147" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B147" s="3" t="s">
         <v>96</v>
@@ -9309,7 +9317,7 @@
     </row>
     <row r="148" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B148" s="3" t="s">
         <v>95</v>
@@ -9321,7 +9329,7 @@
     </row>
     <row r="149" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B149" s="3" t="s">
         <v>92</v>
@@ -9333,7 +9341,7 @@
     </row>
     <row r="150" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B150" s="3" t="s">
         <v>99</v>
@@ -9345,7 +9353,7 @@
     </row>
     <row r="151" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A151" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B151" s="3" t="s">
         <v>64</v>
@@ -9357,7 +9365,7 @@
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B152" s="3" t="s">
         <v>65</v>
@@ -9369,7 +9377,7 @@
     </row>
     <row r="153" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B153" s="3" t="s">
         <v>63</v>
@@ -9381,7 +9389,7 @@
     </row>
     <row r="154" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B154" s="3" t="s">
         <v>11</v>
@@ -9393,7 +9401,7 @@
     </row>
     <row r="155" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B155" s="3" t="s">
         <v>13</v>
@@ -9405,7 +9413,7 @@
     </row>
     <row r="156" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A156" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B156" s="3" t="s">
         <v>9</v>
@@ -9417,7 +9425,7 @@
     </row>
     <row r="157" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B157" s="3" t="s">
         <v>10</v>
@@ -9429,7 +9437,7 @@
     </row>
     <row r="158" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B158" s="3" t="s">
         <v>14</v>
@@ -9441,7 +9449,7 @@
     </row>
     <row r="159" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A159" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B159" s="3" t="s">
         <v>12</v>
@@ -9453,7 +9461,7 @@
     </row>
     <row r="160" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A160" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B160" s="3" t="s">
         <v>8</v>
@@ -9465,7 +9473,7 @@
     </row>
     <row r="161" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A161" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B161" s="3" t="s">
         <v>60</v>
@@ -9477,7 +9485,7 @@
     </row>
     <row r="162" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A162" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B162" s="3" t="s">
         <v>62</v>
@@ -9489,7 +9497,7 @@
     </row>
     <row r="163" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B163" s="3" t="s">
         <v>61</v>
@@ -9501,7 +9509,7 @@
     </row>
     <row r="164" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A164" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B164" s="3" t="s">
         <v>59</v>
@@ -9513,7 +9521,7 @@
     </row>
     <row r="165" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B165" s="3" t="s">
         <v>2</v>
@@ -9525,7 +9533,7 @@
     </row>
     <row r="166" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A166" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B166" s="3" t="s">
         <v>1</v>
@@ -9537,7 +9545,7 @@
     </row>
     <row r="167" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A167" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B167" s="3" t="s">
         <v>3</v>
@@ -9549,7 +9557,7 @@
     </row>
     <row r="168" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A168" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B168" s="3" t="s">
         <v>4</v>
@@ -9561,7 +9569,7 @@
     </row>
     <row r="169" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A169" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B169" s="3" t="s">
         <v>21</v>
@@ -9573,7 +9581,7 @@
     </row>
     <row r="170" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A170" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B170" s="3" t="s">
         <v>23</v>
@@ -9585,7 +9593,7 @@
     </row>
     <row r="171" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A171" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B171" s="3" t="s">
         <v>24</v>
@@ -9597,7 +9605,7 @@
     </row>
     <row r="172" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A172" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B172" s="3" t="s">
         <v>22</v>
@@ -9609,7 +9617,7 @@
     </row>
     <row r="173" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A173" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B173" s="3" t="s">
         <v>40</v>
@@ -9621,7 +9629,7 @@
     </row>
     <row r="174" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A174" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B174" s="3" t="s">
         <v>41</v>
@@ -9633,7 +9641,7 @@
     </row>
     <row r="175" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A175" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B175" s="3" t="s">
         <v>45</v>
@@ -9645,7 +9653,7 @@
     </row>
     <row r="176" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A176" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B176" s="3" t="s">
         <v>42</v>
@@ -9657,7 +9665,7 @@
     </row>
     <row r="177" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A177" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B177" s="3" t="s">
         <v>43</v>
@@ -9669,7 +9677,7 @@
     </row>
     <row r="178" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A178" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B178" s="3" t="s">
         <v>46</v>
@@ -9681,7 +9689,7 @@
     </row>
     <row r="179" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A179" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B179" s="3" t="s">
         <v>48</v>
@@ -9693,7 +9701,7 @@
     </row>
     <row r="180" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A180" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B180" s="3" t="s">
         <v>49</v>
@@ -9705,7 +9713,7 @@
     </row>
     <row r="181" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A181" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B181" s="3" t="s">
         <v>47</v>
@@ -9717,7 +9725,7 @@
     </row>
     <row r="182" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A182" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B182" s="3" t="s">
         <v>44</v>
@@ -9729,7 +9737,7 @@
     </row>
     <row r="183" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A183" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B183" s="3" t="s">
         <v>51</v>
@@ -9741,7 +9749,7 @@
     </row>
     <row r="184" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A184" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B184" s="3" t="s">
         <v>52</v>
@@ -9753,7 +9761,7 @@
     </row>
     <row r="185" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A185" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B185" s="3" t="s">
         <v>55</v>
@@ -9765,7 +9773,7 @@
     </row>
     <row r="186" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A186" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B186" s="3" t="s">
         <v>58</v>
@@ -9777,7 +9785,7 @@
     </row>
     <row r="187" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A187" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B187" s="3" t="s">
         <v>50</v>
@@ -9789,7 +9797,7 @@
     </row>
     <row r="188" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A188" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B188" s="3" t="s">
         <v>56</v>
@@ -9801,7 +9809,7 @@
     </row>
     <row r="189" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A189" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B189" s="3" t="s">
         <v>54</v>
@@ -9813,7 +9821,7 @@
     </row>
     <row r="190" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A190" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B190" s="3" t="s">
         <v>53</v>
@@ -9825,7 +9833,7 @@
     </row>
     <row r="191" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A191" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B191" s="3" t="s">
         <v>57</v>
@@ -9837,7 +9845,7 @@
     </row>
     <row r="192" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A192" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B192" s="3" t="s">
         <v>33</v>
@@ -9849,7 +9857,7 @@
     </row>
     <row r="193" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A193" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B193" s="3" t="s">
         <v>34</v>
@@ -9861,7 +9869,7 @@
     </row>
     <row r="194" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A194" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B194" s="3" t="s">
         <v>70</v>
@@ -9873,7 +9881,7 @@
     </row>
     <row r="195" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A195" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B195" s="3" t="s">
         <v>69</v>
@@ -9885,7 +9893,7 @@
     </row>
     <row r="196" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A196" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B196" s="3" t="s">
         <v>68</v>
@@ -9897,7 +9905,7 @@
     </row>
     <row r="197" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A197" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B197" s="3" t="s">
         <v>37</v>
@@ -9909,7 +9917,7 @@
     </row>
     <row r="198" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A198" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B198" s="3" t="s">
         <v>38</v>
@@ -9921,7 +9929,7 @@
     </row>
     <row r="199" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A199" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B199" s="3" t="s">
         <v>98</v>
@@ -9933,7 +9941,7 @@
     </row>
     <row r="200" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A200" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B200" s="3" t="s">
         <v>97</v>
@@ -9945,7 +9953,7 @@
     </row>
     <row r="201" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A201" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B201" s="3" t="s">
         <v>39</v>
@@ -13557,7 +13565,7 @@
     </row>
     <row r="502" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A502" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B502" s="3" t="s">
         <v>29</v>
@@ -13569,7 +13577,7 @@
     </row>
     <row r="503" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A503" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B503" s="3" t="s">
         <v>83</v>
@@ -13581,7 +13589,7 @@
     </row>
     <row r="504" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A504" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B504" s="3" t="s">
         <v>84</v>
@@ -13593,7 +13601,7 @@
     </row>
     <row r="505" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A505" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B505" s="3" t="s">
         <v>85</v>
@@ -13605,7 +13613,7 @@
     </row>
     <row r="506" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A506" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B506" s="3" t="s">
         <v>86</v>
@@ -13617,7 +13625,7 @@
     </row>
     <row r="507" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A507" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B507" s="3" t="s">
         <v>87</v>
@@ -13629,7 +13637,7 @@
     </row>
     <row r="508" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A508" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B508" s="3" t="s">
         <v>88</v>
@@ -13641,7 +13649,7 @@
     </row>
     <row r="509" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A509" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B509" s="3" t="s">
         <v>25</v>
@@ -13653,7 +13661,7 @@
     </row>
     <row r="510" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A510" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B510" s="3" t="s">
         <v>27</v>
@@ -13665,7 +13673,7 @@
     </row>
     <row r="511" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A511" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B511" s="3" t="s">
         <v>28</v>
@@ -13677,7 +13685,7 @@
     </row>
     <row r="512" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A512" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B512" s="3" t="s">
         <v>26</v>
@@ -13689,7 +13697,7 @@
     </row>
     <row r="513" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A513" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B513" s="3" t="s">
         <v>36</v>
@@ -13701,7 +13709,7 @@
     </row>
     <row r="514" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A514" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B514" s="3" t="s">
         <v>35</v>
@@ -13713,7 +13721,7 @@
     </row>
     <row r="515" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A515" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B515" s="3" t="s">
         <v>5</v>
@@ -13725,7 +13733,7 @@
     </row>
     <row r="516" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A516" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B516" s="3" t="s">
         <v>6</v>
@@ -13737,7 +13745,7 @@
     </row>
     <row r="517" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A517" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B517" s="3" t="s">
         <v>7</v>
@@ -13749,7 +13757,7 @@
     </row>
     <row r="518" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A518" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B518" s="3" t="s">
         <v>31</v>
@@ -13761,7 +13769,7 @@
     </row>
     <row r="519" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A519" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B519" s="3" t="s">
         <v>32</v>
@@ -13773,7 +13781,7 @@
     </row>
     <row r="520" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A520" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B520" s="3" t="s">
         <v>30</v>
@@ -13785,7 +13793,7 @@
     </row>
     <row r="521" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A521" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B521" s="3" t="s">
         <v>100</v>
@@ -13797,7 +13805,7 @@
     </row>
     <row r="522" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A522" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B522" s="3" t="s">
         <v>67</v>
@@ -13809,7 +13817,7 @@
     </row>
     <row r="523" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A523" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B523" s="3" t="s">
         <v>66</v>
@@ -13821,7 +13829,7 @@
     </row>
     <row r="524" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A524" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B524" s="3" t="s">
         <v>78</v>
@@ -13833,7 +13841,7 @@
     </row>
     <row r="525" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A525" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B525" s="3" t="s">
         <v>79</v>
@@ -13845,7 +13853,7 @@
     </row>
     <row r="526" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A526" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B526" s="3" t="s">
         <v>71</v>
@@ -13857,7 +13865,7 @@
     </row>
     <row r="527" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A527" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B527" s="3" t="s">
         <v>72</v>
@@ -13869,7 +13877,7 @@
     </row>
     <row r="528" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A528" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B528" s="3" t="s">
         <v>81</v>
@@ -13881,7 +13889,7 @@
     </row>
     <row r="529" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A529" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B529" s="3" t="s">
         <v>74</v>
@@ -13893,7 +13901,7 @@
     </row>
     <row r="530" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A530" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B530" s="3" t="s">
         <v>73</v>
@@ -13905,7 +13913,7 @@
     </row>
     <row r="531" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A531" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B531" s="3" t="s">
         <v>75</v>
@@ -13917,7 +13925,7 @@
     </row>
     <row r="532" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A532" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B532" s="3" t="s">
         <v>82</v>
@@ -13929,7 +13937,7 @@
     </row>
     <row r="533" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A533" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B533" s="3" t="s">
         <v>80</v>
@@ -13941,7 +13949,7 @@
     </row>
     <row r="534" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A534" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B534" s="3" t="s">
         <v>76</v>
@@ -13953,7 +13961,7 @@
     </row>
     <row r="535" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A535" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B535" s="3" t="s">
         <v>77</v>
@@ -13965,7 +13973,7 @@
     </row>
     <row r="536" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A536" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B536" s="3" t="s">
         <v>15</v>
@@ -13977,7 +13985,7 @@
     </row>
     <row r="537" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A537" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B537" s="3" t="s">
         <v>17</v>
@@ -13989,7 +13997,7 @@
     </row>
     <row r="538" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A538" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B538" s="3" t="s">
         <v>16</v>
@@ -14001,7 +14009,7 @@
     </row>
     <row r="539" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A539" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B539" s="3" t="s">
         <v>19</v>
@@ -14013,7 +14021,7 @@
     </row>
     <row r="540" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A540" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B540" s="3" t="s">
         <v>18</v>
@@ -14025,7 +14033,7 @@
     </row>
     <row r="541" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A541" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B541" s="3" t="s">
         <v>20</v>
@@ -14037,7 +14045,7 @@
     </row>
     <row r="542" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A542" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B542" s="3" t="s">
         <v>90</v>
@@ -14049,7 +14057,7 @@
     </row>
     <row r="543" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A543" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B543" s="3" t="s">
         <v>89</v>
@@ -14061,7 +14069,7 @@
     </row>
     <row r="544" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A544" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B544" s="3" t="s">
         <v>93</v>
@@ -14073,7 +14081,7 @@
     </row>
     <row r="545" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A545" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B545" s="3" t="s">
         <v>94</v>
@@ -14085,7 +14093,7 @@
     </row>
     <row r="546" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A546" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B546" s="3" t="s">
         <v>91</v>
@@ -14097,7 +14105,7 @@
     </row>
     <row r="547" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A547" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B547" s="3" t="s">
         <v>96</v>
@@ -14109,7 +14117,7 @@
     </row>
     <row r="548" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A548" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B548" s="3" t="s">
         <v>95</v>
@@ -14121,7 +14129,7 @@
     </row>
     <row r="549" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A549" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B549" s="3" t="s">
         <v>92</v>
@@ -14133,7 +14141,7 @@
     </row>
     <row r="550" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A550" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B550" s="3" t="s">
         <v>99</v>
@@ -14145,7 +14153,7 @@
     </row>
     <row r="551" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A551" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B551" s="3" t="s">
         <v>64</v>
@@ -14157,7 +14165,7 @@
     </row>
     <row r="552" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A552" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B552" s="3" t="s">
         <v>65</v>
@@ -14169,7 +14177,7 @@
     </row>
     <row r="553" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A553" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B553" s="3" t="s">
         <v>63</v>
@@ -14181,7 +14189,7 @@
     </row>
     <row r="554" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A554" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B554" s="3" t="s">
         <v>11</v>
@@ -14193,7 +14201,7 @@
     </row>
     <row r="555" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A555" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B555" s="3" t="s">
         <v>13</v>
@@ -14205,7 +14213,7 @@
     </row>
     <row r="556" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A556" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B556" s="3" t="s">
         <v>9</v>
@@ -14217,7 +14225,7 @@
     </row>
     <row r="557" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A557" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B557" s="3" t="s">
         <v>10</v>
@@ -14229,7 +14237,7 @@
     </row>
     <row r="558" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A558" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B558" s="3" t="s">
         <v>14</v>
@@ -14241,7 +14249,7 @@
     </row>
     <row r="559" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A559" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B559" s="3" t="s">
         <v>12</v>
@@ -14253,7 +14261,7 @@
     </row>
     <row r="560" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A560" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B560" s="3" t="s">
         <v>8</v>
@@ -14265,7 +14273,7 @@
     </row>
     <row r="561" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A561" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B561" s="3" t="s">
         <v>60</v>
@@ -14277,7 +14285,7 @@
     </row>
     <row r="562" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A562" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B562" s="3" t="s">
         <v>62</v>
@@ -14289,7 +14297,7 @@
     </row>
     <row r="563" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A563" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B563" s="3" t="s">
         <v>61</v>
@@ -14301,7 +14309,7 @@
     </row>
     <row r="564" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A564" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B564" s="3" t="s">
         <v>59</v>
@@ -14313,7 +14321,7 @@
     </row>
     <row r="565" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A565" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B565" s="3" t="s">
         <v>2</v>
@@ -14325,7 +14333,7 @@
     </row>
     <row r="566" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A566" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B566" s="3" t="s">
         <v>1</v>
@@ -14337,7 +14345,7 @@
     </row>
     <row r="567" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A567" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B567" s="3" t="s">
         <v>3</v>
@@ -14349,7 +14357,7 @@
     </row>
     <row r="568" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A568" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B568" s="3" t="s">
         <v>4</v>
@@ -14361,7 +14369,7 @@
     </row>
     <row r="569" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A569" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B569" s="3" t="s">
         <v>21</v>
@@ -14373,7 +14381,7 @@
     </row>
     <row r="570" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A570" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B570" s="3" t="s">
         <v>23</v>
@@ -14385,7 +14393,7 @@
     </row>
     <row r="571" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A571" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B571" s="3" t="s">
         <v>24</v>
@@ -14397,7 +14405,7 @@
     </row>
     <row r="572" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A572" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B572" s="3" t="s">
         <v>22</v>
@@ -14409,7 +14417,7 @@
     </row>
     <row r="573" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A573" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B573" s="3" t="s">
         <v>40</v>
@@ -14421,7 +14429,7 @@
     </row>
     <row r="574" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A574" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B574" s="3" t="s">
         <v>41</v>
@@ -14433,7 +14441,7 @@
     </row>
     <row r="575" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A575" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B575" s="3" t="s">
         <v>45</v>
@@ -14445,7 +14453,7 @@
     </row>
     <row r="576" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A576" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B576" s="3" t="s">
         <v>42</v>
@@ -14457,7 +14465,7 @@
     </row>
     <row r="577" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A577" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B577" s="3" t="s">
         <v>43</v>
@@ -14469,7 +14477,7 @@
     </row>
     <row r="578" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A578" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B578" s="3" t="s">
         <v>46</v>
@@ -14481,7 +14489,7 @@
     </row>
     <row r="579" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A579" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B579" s="3" t="s">
         <v>48</v>
@@ -14493,7 +14501,7 @@
     </row>
     <row r="580" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A580" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B580" s="3" t="s">
         <v>49</v>
@@ -14505,7 +14513,7 @@
     </row>
     <row r="581" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A581" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B581" s="3" t="s">
         <v>47</v>
@@ -14517,7 +14525,7 @@
     </row>
     <row r="582" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A582" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B582" s="3" t="s">
         <v>44</v>
@@ -14529,7 +14537,7 @@
     </row>
     <row r="583" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A583" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B583" s="3" t="s">
         <v>51</v>
@@ -14541,7 +14549,7 @@
     </row>
     <row r="584" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A584" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B584" s="3" t="s">
         <v>52</v>
@@ -14553,7 +14561,7 @@
     </row>
     <row r="585" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A585" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B585" s="3" t="s">
         <v>55</v>
@@ -14565,7 +14573,7 @@
     </row>
     <row r="586" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A586" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B586" s="3" t="s">
         <v>58</v>
@@ -14577,7 +14585,7 @@
     </row>
     <row r="587" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A587" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B587" s="3" t="s">
         <v>50</v>
@@ -14589,7 +14597,7 @@
     </row>
     <row r="588" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A588" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B588" s="3" t="s">
         <v>56</v>
@@ -14601,7 +14609,7 @@
     </row>
     <row r="589" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A589" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B589" s="3" t="s">
         <v>54</v>
@@ -14613,7 +14621,7 @@
     </row>
     <row r="590" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A590" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B590" s="3" t="s">
         <v>53</v>
@@ -14625,7 +14633,7 @@
     </row>
     <row r="591" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A591" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B591" s="3" t="s">
         <v>57</v>
@@ -14637,7 +14645,7 @@
     </row>
     <row r="592" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A592" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B592" s="3" t="s">
         <v>33</v>
@@ -14649,7 +14657,7 @@
     </row>
     <row r="593" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A593" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B593" s="3" t="s">
         <v>34</v>
@@ -14661,7 +14669,7 @@
     </row>
     <row r="594" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A594" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B594" s="3" t="s">
         <v>70</v>
@@ -14673,7 +14681,7 @@
     </row>
     <row r="595" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A595" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B595" s="3" t="s">
         <v>69</v>
@@ -14685,7 +14693,7 @@
     </row>
     <row r="596" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A596" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B596" s="3" t="s">
         <v>68</v>
@@ -14697,7 +14705,7 @@
     </row>
     <row r="597" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A597" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B597" s="3" t="s">
         <v>37</v>
@@ -14709,7 +14717,7 @@
     </row>
     <row r="598" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A598" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B598" s="3" t="s">
         <v>38</v>
@@ -14721,7 +14729,7 @@
     </row>
     <row r="599" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A599" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B599" s="3" t="s">
         <v>98</v>
@@ -14733,7 +14741,7 @@
     </row>
     <row r="600" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A600" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B600" s="3" t="s">
         <v>97</v>
@@ -14745,7 +14753,7 @@
     </row>
     <row r="601" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A601" s="3" t="s">
-        <v>128</v>
+        <v>120</v>
       </c>
       <c r="B601" s="3" t="s">
         <v>39</v>
@@ -14756,7 +14764,7 @@
       </c>
     </row>
   </sheetData>
-  <phoneticPr fontId="8" type="noConversion"/>
+  <phoneticPr fontId="9" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -14783,12 +14791,12 @@
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>29</v>
@@ -14800,7 +14808,7 @@
     </row>
     <row r="3" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>83</v>
@@ -14812,7 +14820,7 @@
     </row>
     <row r="4" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>84</v>
@@ -14824,7 +14832,7 @@
     </row>
     <row r="5" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>85</v>
@@ -14836,7 +14844,7 @@
     </row>
     <row r="6" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>86</v>
@@ -14848,7 +14856,7 @@
     </row>
     <row r="7" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>87</v>
@@ -14860,7 +14868,7 @@
     </row>
     <row r="8" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>88</v>
@@ -14872,7 +14880,7 @@
     </row>
     <row r="9" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>25</v>
@@ -14884,7 +14892,7 @@
     </row>
     <row r="10" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>27</v>
@@ -14896,7 +14904,7 @@
     </row>
     <row r="11" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>28</v>
@@ -14908,7 +14916,7 @@
     </row>
     <row r="12" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>26</v>
@@ -14920,7 +14928,7 @@
     </row>
     <row r="13" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>36</v>
@@ -14932,7 +14940,7 @@
     </row>
     <row r="14" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>35</v>
@@ -14944,7 +14952,7 @@
     </row>
     <row r="15" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>5</v>
@@ -14956,7 +14964,7 @@
     </row>
     <row r="16" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>6</v>
@@ -14968,7 +14976,7 @@
     </row>
     <row r="17" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>7</v>
@@ -14980,7 +14988,7 @@
     </row>
     <row r="18" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>31</v>
@@ -14992,7 +15000,7 @@
     </row>
     <row r="19" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>32</v>
@@ -15004,7 +15012,7 @@
     </row>
     <row r="20" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>30</v>
@@ -15016,7 +15024,7 @@
     </row>
     <row r="21" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>100</v>
@@ -15028,7 +15036,7 @@
     </row>
     <row r="22" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>67</v>
@@ -15040,7 +15048,7 @@
     </row>
     <row r="23" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>66</v>
@@ -15052,7 +15060,7 @@
     </row>
     <row r="24" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>78</v>
@@ -15064,7 +15072,7 @@
     </row>
     <row r="25" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>79</v>
@@ -15076,7 +15084,7 @@
     </row>
     <row r="26" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>71</v>
@@ -15088,7 +15096,7 @@
     </row>
     <row r="27" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>72</v>
@@ -15100,7 +15108,7 @@
     </row>
     <row r="28" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>81</v>
@@ -15112,7 +15120,7 @@
     </row>
     <row r="29" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>74</v>
@@ -15124,7 +15132,7 @@
     </row>
     <row r="30" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>73</v>
@@ -15136,7 +15144,7 @@
     </row>
     <row r="31" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>75</v>
@@ -15148,7 +15156,7 @@
     </row>
     <row r="32" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>82</v>
@@ -15160,7 +15168,7 @@
     </row>
     <row r="33" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>80</v>
@@ -15172,7 +15180,7 @@
     </row>
     <row r="34" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>76</v>
@@ -15184,7 +15192,7 @@
     </row>
     <row r="35" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B35" s="1" t="s">
         <v>77</v>
@@ -15196,7 +15204,7 @@
     </row>
     <row r="36" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>15</v>
@@ -15208,7 +15216,7 @@
     </row>
     <row r="37" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B37" s="1" t="s">
         <v>17</v>
@@ -15220,7 +15228,7 @@
     </row>
     <row r="38" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B38" s="1" t="s">
         <v>16</v>
@@ -15232,7 +15240,7 @@
     </row>
     <row r="39" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>19</v>
@@ -15244,7 +15252,7 @@
     </row>
     <row r="40" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B40" s="1" t="s">
         <v>18</v>
@@ -15256,7 +15264,7 @@
     </row>
     <row r="41" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B41" s="1" t="s">
         <v>20</v>
@@ -15268,7 +15276,7 @@
     </row>
     <row r="42" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>90</v>
@@ -15280,7 +15288,7 @@
     </row>
     <row r="43" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B43" s="1" t="s">
         <v>89</v>
@@ -15292,7 +15300,7 @@
     </row>
     <row r="44" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>93</v>
@@ -15304,7 +15312,7 @@
     </row>
     <row r="45" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>94</v>
@@ -15316,7 +15324,7 @@
     </row>
     <row r="46" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>91</v>
@@ -15328,7 +15336,7 @@
     </row>
     <row r="47" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>96</v>
@@ -15340,7 +15348,7 @@
     </row>
     <row r="48" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B48" s="1" t="s">
         <v>95</v>
@@ -15352,7 +15360,7 @@
     </row>
     <row r="49" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>92</v>
@@ -15364,7 +15372,7 @@
     </row>
     <row r="50" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A50" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>99</v>
@@ -15376,7 +15384,7 @@
     </row>
     <row r="51" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A51" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>64</v>
@@ -15388,7 +15396,7 @@
     </row>
     <row r="52" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A52" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>65</v>
@@ -15400,7 +15408,7 @@
     </row>
     <row r="53" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A53" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>63</v>
@@ -15412,7 +15420,7 @@
     </row>
     <row r="54" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A54" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>11</v>
@@ -15424,7 +15432,7 @@
     </row>
     <row r="55" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A55" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>13</v>
@@ -15436,7 +15444,7 @@
     </row>
     <row r="56" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A56" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>9</v>
@@ -15448,7 +15456,7 @@
     </row>
     <row r="57" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A57" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>10</v>
@@ -15460,7 +15468,7 @@
     </row>
     <row r="58" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A58" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>14</v>
@@ -15472,7 +15480,7 @@
     </row>
     <row r="59" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A59" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>12</v>
@@ -15484,7 +15492,7 @@
     </row>
     <row r="60" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A60" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>8</v>
@@ -15496,7 +15504,7 @@
     </row>
     <row r="61" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A61" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B61" s="1" t="s">
         <v>60</v>
@@ -15508,7 +15516,7 @@
     </row>
     <row r="62" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A62" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B62" s="1" t="s">
         <v>62</v>
@@ -15520,7 +15528,7 @@
     </row>
     <row r="63" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A63" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>61</v>
@@ -15532,7 +15540,7 @@
     </row>
     <row r="64" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A64" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>59</v>
@@ -15544,7 +15552,7 @@
     </row>
     <row r="65" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A65" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>2</v>
@@ -15556,7 +15564,7 @@
     </row>
     <row r="66" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A66" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>1</v>
@@ -15568,7 +15576,7 @@
     </row>
     <row r="67" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A67" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>3</v>
@@ -15580,7 +15588,7 @@
     </row>
     <row r="68" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A68" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B68" s="1" t="s">
         <v>4</v>
@@ -15592,7 +15600,7 @@
     </row>
     <row r="69" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A69" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B69" s="1" t="s">
         <v>21</v>
@@ -15604,7 +15612,7 @@
     </row>
     <row r="70" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A70" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B70" s="1" t="s">
         <v>23</v>
@@ -15616,7 +15624,7 @@
     </row>
     <row r="71" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A71" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>24</v>
@@ -15628,7 +15636,7 @@
     </row>
     <row r="72" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A72" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>22</v>
@@ -15640,7 +15648,7 @@
     </row>
     <row r="73" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A73" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B73" s="1" t="s">
         <v>40</v>
@@ -15652,7 +15660,7 @@
     </row>
     <row r="74" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A74" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>41</v>
@@ -15664,7 +15672,7 @@
     </row>
     <row r="75" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A75" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B75" s="1" t="s">
         <v>45</v>
@@ -15676,7 +15684,7 @@
     </row>
     <row r="76" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A76" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>42</v>
@@ -15688,7 +15696,7 @@
     </row>
     <row r="77" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A77" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B77" s="1" t="s">
         <v>43</v>
@@ -15700,7 +15708,7 @@
     </row>
     <row r="78" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A78" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>46</v>
@@ -15712,7 +15720,7 @@
     </row>
     <row r="79" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A79" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>48</v>
@@ -15724,7 +15732,7 @@
     </row>
     <row r="80" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A80" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B80" s="1" t="s">
         <v>49</v>
@@ -15736,7 +15744,7 @@
     </row>
     <row r="81" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A81" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>47</v>
@@ -15748,7 +15756,7 @@
     </row>
     <row r="82" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A82" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>44</v>
@@ -15760,7 +15768,7 @@
     </row>
     <row r="83" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A83" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>51</v>
@@ -15772,7 +15780,7 @@
     </row>
     <row r="84" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A84" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>52</v>
@@ -15784,7 +15792,7 @@
     </row>
     <row r="85" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A85" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>55</v>
@@ -15796,7 +15804,7 @@
     </row>
     <row r="86" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A86" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>58</v>
@@ -15808,7 +15816,7 @@
     </row>
     <row r="87" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A87" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>50</v>
@@ -15820,7 +15828,7 @@
     </row>
     <row r="88" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A88" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B88" s="1" t="s">
         <v>56</v>
@@ -15832,7 +15840,7 @@
     </row>
     <row r="89" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A89" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B89" s="1" t="s">
         <v>54</v>
@@ -15844,7 +15852,7 @@
     </row>
     <row r="90" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A90" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B90" s="1" t="s">
         <v>53</v>
@@ -15856,7 +15864,7 @@
     </row>
     <row r="91" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A91" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>57</v>
@@ -15868,7 +15876,7 @@
     </row>
     <row r="92" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A92" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>33</v>
@@ -15880,7 +15888,7 @@
     </row>
     <row r="93" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A93" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>34</v>
@@ -15892,7 +15900,7 @@
     </row>
     <row r="94" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A94" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>70</v>
@@ -15904,7 +15912,7 @@
     </row>
     <row r="95" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A95" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>69</v>
@@ -15916,7 +15924,7 @@
     </row>
     <row r="96" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A96" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>68</v>
@@ -15928,7 +15936,7 @@
     </row>
     <row r="97" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A97" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B97" s="1" t="s">
         <v>37</v>
@@ -15940,7 +15948,7 @@
     </row>
     <row r="98" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A98" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B98" s="1" t="s">
         <v>38</v>
@@ -15952,7 +15960,7 @@
     </row>
     <row r="99" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A99" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>98</v>
@@ -15964,7 +15972,7 @@
     </row>
     <row r="100" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A100" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>97</v>
@@ -15976,7 +15984,7 @@
     </row>
     <row r="101" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A101" s="5" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B101" s="1" t="s">
         <v>39</v>
@@ -15988,7 +15996,7 @@
     </row>
     <row r="102" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A102" s="8" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B102" s="1" t="s">
         <v>29</v>
@@ -16000,7 +16008,7 @@
     </row>
     <row r="103" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A103" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B103" s="1" t="s">
         <v>83</v>
@@ -16012,7 +16020,7 @@
     </row>
     <row r="104" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A104" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B104" s="1" t="s">
         <v>84</v>
@@ -16024,7 +16032,7 @@
     </row>
     <row r="105" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A105" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B105" s="1" t="s">
         <v>85</v>
@@ -16036,7 +16044,7 @@
     </row>
     <row r="106" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A106" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B106" s="1" t="s">
         <v>86</v>
@@ -16048,7 +16056,7 @@
     </row>
     <row r="107" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A107" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B107" s="1" t="s">
         <v>87</v>
@@ -16060,7 +16068,7 @@
     </row>
     <row r="108" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A108" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B108" s="1" t="s">
         <v>88</v>
@@ -16072,7 +16080,7 @@
     </row>
     <row r="109" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A109" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B109" s="1" t="s">
         <v>25</v>
@@ -16084,7 +16092,7 @@
     </row>
     <row r="110" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A110" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B110" s="1" t="s">
         <v>27</v>
@@ -16096,7 +16104,7 @@
     </row>
     <row r="111" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A111" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B111" s="1" t="s">
         <v>28</v>
@@ -16108,7 +16116,7 @@
     </row>
     <row r="112" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A112" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B112" s="1" t="s">
         <v>26</v>
@@ -16120,7 +16128,7 @@
     </row>
     <row r="113" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A113" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B113" s="1" t="s">
         <v>36</v>
@@ -16132,7 +16140,7 @@
     </row>
     <row r="114" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A114" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B114" s="1" t="s">
         <v>35</v>
@@ -16144,7 +16152,7 @@
     </row>
     <row r="115" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A115" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B115" s="1" t="s">
         <v>5</v>
@@ -16156,7 +16164,7 @@
     </row>
     <row r="116" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A116" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B116" s="1" t="s">
         <v>6</v>
@@ -16168,7 +16176,7 @@
     </row>
     <row r="117" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A117" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B117" s="1" t="s">
         <v>7</v>
@@ -16180,7 +16188,7 @@
     </row>
     <row r="118" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A118" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B118" s="1" t="s">
         <v>31</v>
@@ -16192,7 +16200,7 @@
     </row>
     <row r="119" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A119" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B119" s="1" t="s">
         <v>32</v>
@@ -16204,7 +16212,7 @@
     </row>
     <row r="120" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A120" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B120" s="1" t="s">
         <v>30</v>
@@ -16216,7 +16224,7 @@
     </row>
     <row r="121" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A121" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B121" s="1" t="s">
         <v>100</v>
@@ -16228,7 +16236,7 @@
     </row>
     <row r="122" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A122" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B122" s="1" t="s">
         <v>67</v>
@@ -16240,7 +16248,7 @@
     </row>
     <row r="123" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A123" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B123" s="1" t="s">
         <v>66</v>
@@ -16252,7 +16260,7 @@
     </row>
     <row r="124" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A124" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B124" s="1" t="s">
         <v>78</v>
@@ -16264,7 +16272,7 @@
     </row>
     <row r="125" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A125" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B125" s="1" t="s">
         <v>79</v>
@@ -16276,7 +16284,7 @@
     </row>
     <row r="126" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A126" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>71</v>
@@ -16288,7 +16296,7 @@
     </row>
     <row r="127" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A127" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B127" s="1" t="s">
         <v>72</v>
@@ -16300,7 +16308,7 @@
     </row>
     <row r="128" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A128" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B128" s="1" t="s">
         <v>81</v>
@@ -16312,7 +16320,7 @@
     </row>
     <row r="129" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A129" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B129" s="1" t="s">
         <v>74</v>
@@ -16324,7 +16332,7 @@
     </row>
     <row r="130" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A130" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B130" s="1" t="s">
         <v>73</v>
@@ -16336,7 +16344,7 @@
     </row>
     <row r="131" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A131" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>75</v>
@@ -16348,7 +16356,7 @@
     </row>
     <row r="132" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A132" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B132" s="1" t="s">
         <v>82</v>
@@ -16360,7 +16368,7 @@
     </row>
     <row r="133" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A133" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B133" s="1" t="s">
         <v>80</v>
@@ -16372,7 +16380,7 @@
     </row>
     <row r="134" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A134" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B134" s="1" t="s">
         <v>76</v>
@@ -16384,7 +16392,7 @@
     </row>
     <row r="135" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A135" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>77</v>
@@ -16396,7 +16404,7 @@
     </row>
     <row r="136" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A136" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B136" s="1" t="s">
         <v>15</v>
@@ -16408,7 +16416,7 @@
     </row>
     <row r="137" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A137" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>17</v>
@@ -16420,7 +16428,7 @@
     </row>
     <row r="138" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A138" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B138" s="1" t="s">
         <v>16</v>
@@ -16432,7 +16440,7 @@
     </row>
     <row r="139" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A139" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>19</v>
@@ -16444,7 +16452,7 @@
     </row>
     <row r="140" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A140" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B140" s="1" t="s">
         <v>18</v>
@@ -16456,7 +16464,7 @@
     </row>
     <row r="141" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A141" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B141" s="1" t="s">
         <v>20</v>
@@ -16468,7 +16476,7 @@
     </row>
     <row r="142" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A142" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B142" s="1" t="s">
         <v>90</v>
@@ -16480,7 +16488,7 @@
     </row>
     <row r="143" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A143" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B143" s="1" t="s">
         <v>89</v>
@@ -16492,7 +16500,7 @@
     </row>
     <row r="144" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A144" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B144" s="1" t="s">
         <v>93</v>
@@ -16504,7 +16512,7 @@
     </row>
     <row r="145" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A145" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B145" s="1" t="s">
         <v>94</v>
@@ -16516,7 +16524,7 @@
     </row>
     <row r="146" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A146" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B146" s="1" t="s">
         <v>91</v>
@@ -16528,7 +16536,7 @@
     </row>
     <row r="147" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A147" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>96</v>
@@ -16540,7 +16548,7 @@
     </row>
     <row r="148" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A148" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B148" s="1" t="s">
         <v>95</v>
@@ -16552,7 +16560,7 @@
     </row>
     <row r="149" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A149" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B149" s="1" t="s">
         <v>92</v>
@@ -16564,7 +16572,7 @@
     </row>
     <row r="150" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A150" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B150" s="1" t="s">
         <v>99</v>
@@ -16576,7 +16584,7 @@
     </row>
     <row r="151" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A151" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B151" s="1" t="s">
         <v>64</v>
@@ -16588,7 +16596,7 @@
     </row>
     <row r="152" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A152" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>65</v>
@@ -16600,7 +16608,7 @@
     </row>
     <row r="153" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A153" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>63</v>
@@ -16612,7 +16620,7 @@
     </row>
     <row r="154" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A154" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>11</v>
@@ -16624,7 +16632,7 @@
     </row>
     <row r="155" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A155" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>13</v>
@@ -16636,7 +16644,7 @@
     </row>
     <row r="156" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A156" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>9</v>
@@ -16648,7 +16656,7 @@
     </row>
     <row r="157" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A157" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B157" s="1" t="s">
         <v>10</v>
@@ -16660,7 +16668,7 @@
     </row>
     <row r="158" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A158" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B158" s="1" t="s">
         <v>14</v>
@@ -16672,7 +16680,7 @@
     </row>
     <row r="159" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A159" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B159" s="1" t="s">
         <v>12</v>
@@ -16684,7 +16692,7 @@
     </row>
     <row r="160" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A160" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B160" s="1" t="s">
         <v>8</v>
@@ -16696,7 +16704,7 @@
     </row>
     <row r="161" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A161" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B161" s="1" t="s">
         <v>60</v>
@@ -16708,7 +16716,7 @@
     </row>
     <row r="162" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A162" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B162" s="1" t="s">
         <v>62</v>
@@ -16720,7 +16728,7 @@
     </row>
     <row r="163" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A163" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B163" s="1" t="s">
         <v>61</v>
@@ -16732,7 +16740,7 @@
     </row>
     <row r="164" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A164" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B164" s="1" t="s">
         <v>59</v>
@@ -16744,7 +16752,7 @@
     </row>
     <row r="165" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A165" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B165" s="1" t="s">
         <v>2</v>
@@ -16756,7 +16764,7 @@
     </row>
     <row r="166" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A166" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B166" s="1" t="s">
         <v>1</v>
@@ -16768,7 +16776,7 @@
     </row>
     <row r="167" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A167" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B167" s="1" t="s">
         <v>3</v>
@@ -16780,7 +16788,7 @@
     </row>
     <row r="168" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A168" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B168" s="1" t="s">
         <v>4</v>
@@ -16792,7 +16800,7 @@
     </row>
     <row r="169" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A169" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B169" s="1" t="s">
         <v>21</v>
@@ -16804,7 +16812,7 @@
     </row>
     <row r="170" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A170" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B170" s="1" t="s">
         <v>23</v>
@@ -16816,7 +16824,7 @@
     </row>
     <row r="171" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A171" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B171" s="1" t="s">
         <v>24</v>
@@ -16828,7 +16836,7 @@
     </row>
     <row r="172" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A172" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B172" s="1" t="s">
         <v>22</v>
@@ -16840,7 +16848,7 @@
     </row>
     <row r="173" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A173" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B173" s="1" t="s">
         <v>40</v>
@@ -16852,7 +16860,7 @@
     </row>
     <row r="174" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A174" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B174" s="1" t="s">
         <v>41</v>
@@ -16864,7 +16872,7 @@
     </row>
     <row r="175" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A175" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B175" s="1" t="s">
         <v>45</v>
@@ -16876,7 +16884,7 @@
     </row>
     <row r="176" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A176" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B176" s="1" t="s">
         <v>42</v>
@@ -16888,7 +16896,7 @@
     </row>
     <row r="177" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A177" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B177" s="1" t="s">
         <v>43</v>
@@ -16900,7 +16908,7 @@
     </row>
     <row r="178" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A178" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B178" s="1" t="s">
         <v>46</v>
@@ -16912,7 +16920,7 @@
     </row>
     <row r="179" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A179" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B179" s="1" t="s">
         <v>48</v>
@@ -16924,7 +16932,7 @@
     </row>
     <row r="180" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A180" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B180" s="1" t="s">
         <v>49</v>
@@ -16936,7 +16944,7 @@
     </row>
     <row r="181" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A181" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B181" s="1" t="s">
         <v>47</v>
@@ -16948,7 +16956,7 @@
     </row>
     <row r="182" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A182" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B182" s="1" t="s">
         <v>44</v>
@@ -16960,7 +16968,7 @@
     </row>
     <row r="183" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A183" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B183" s="1" t="s">
         <v>51</v>
@@ -16972,7 +16980,7 @@
     </row>
     <row r="184" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A184" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B184" s="1" t="s">
         <v>52</v>
@@ -16984,7 +16992,7 @@
     </row>
     <row r="185" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A185" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B185" s="1" t="s">
         <v>55</v>
@@ -16996,7 +17004,7 @@
     </row>
     <row r="186" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A186" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B186" s="1" t="s">
         <v>58</v>
@@ -17008,7 +17016,7 @@
     </row>
     <row r="187" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A187" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B187" s="1" t="s">
         <v>50</v>
@@ -17020,7 +17028,7 @@
     </row>
     <row r="188" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A188" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B188" s="1" t="s">
         <v>56</v>
@@ -17032,7 +17040,7 @@
     </row>
     <row r="189" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A189" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B189" s="1" t="s">
         <v>54</v>
@@ -17044,7 +17052,7 @@
     </row>
     <row r="190" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A190" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B190" s="1" t="s">
         <v>53</v>
@@ -17056,7 +17064,7 @@
     </row>
     <row r="191" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A191" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B191" s="1" t="s">
         <v>57</v>
@@ -17068,7 +17076,7 @@
     </row>
     <row r="192" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A192" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B192" s="1" t="s">
         <v>33</v>
@@ -17080,7 +17088,7 @@
     </row>
     <row r="193" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A193" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B193" s="1" t="s">
         <v>34</v>
@@ -17092,7 +17100,7 @@
     </row>
     <row r="194" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A194" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B194" s="1" t="s">
         <v>70</v>
@@ -17104,7 +17112,7 @@
     </row>
     <row r="195" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A195" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B195" s="1" t="s">
         <v>69</v>
@@ -17116,7 +17124,7 @@
     </row>
     <row r="196" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A196" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B196" s="1" t="s">
         <v>68</v>
@@ -17128,7 +17136,7 @@
     </row>
     <row r="197" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A197" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B197" s="1" t="s">
         <v>37</v>
@@ -17140,7 +17148,7 @@
     </row>
     <row r="198" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A198" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B198" s="1" t="s">
         <v>38</v>
@@ -17152,7 +17160,7 @@
     </row>
     <row r="199" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A199" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B199" s="1" t="s">
         <v>98</v>
@@ -17164,7 +17172,7 @@
     </row>
     <row r="200" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A200" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B200" s="1" t="s">
         <v>97</v>
@@ -17176,7 +17184,7 @@
     </row>
     <row r="201" spans="1:3" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A201" s="4" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B201" s="1" t="s">
         <v>39</v>

</xml_diff>